<commit_message>
Atualização de CodeSystems e ValueSet
</commit_message>
<xml_diff>
--- a/output/CodeSystem-BRNomeExameGAL.xlsx
+++ b/output/CodeSystem-BRNomeExameGAL.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="160">
   <si>
     <t>Property</t>
   </si>
@@ -418,6 +418,81 @@
   </si>
   <si>
     <t>Vírus Respiratórios</t>
+  </si>
+  <si>
+    <t>BORDT</t>
+  </si>
+  <si>
+    <t>Bordetella</t>
+  </si>
+  <si>
+    <t>BORID</t>
+  </si>
+  <si>
+    <t>Bordetella, Identificação</t>
+  </si>
+  <si>
+    <t>COQBM</t>
+  </si>
+  <si>
+    <t>Coqueluche, Detecção de Bordetella pertussis</t>
+  </si>
+  <si>
+    <t>COQCU</t>
+  </si>
+  <si>
+    <t>BORDTA</t>
+  </si>
+  <si>
+    <t>Coqueluche, IgA</t>
+  </si>
+  <si>
+    <t>BORDTG</t>
+  </si>
+  <si>
+    <t>Coqueluche, IgG</t>
+  </si>
+  <si>
+    <t>COQGRT</t>
+  </si>
+  <si>
+    <t>Coqueluche, Pesquisa de Genes de Resistência</t>
+  </si>
+  <si>
+    <t>COQSR</t>
+  </si>
+  <si>
+    <t>Coqueluche, Sorologia</t>
+  </si>
+  <si>
+    <t>DIFCU</t>
+  </si>
+  <si>
+    <t>Difteria, Cultura</t>
+  </si>
+  <si>
+    <t>DIFGEN</t>
+  </si>
+  <si>
+    <t>Difteria, Pesquisa de genes</t>
+  </si>
+  <si>
+    <t>COCUL</t>
+  </si>
+  <si>
+    <t>Cólera</t>
+  </si>
+  <si>
+    <t>COLBM</t>
+  </si>
+  <si>
+    <t>Cólera, Biologia Molecular</t>
+  </si>
+  <si>
+    <t>COTSA</t>
+  </si>
+  <si>
+    <t>Cólera, Teste de Sensibilidade</t>
   </si>
 </sst>
 </file>
@@ -725,7 +800,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1306,6 +1381,162 @@
       </c>
       <c r="D48" s="2"/>
     </row>
+    <row r="49">
+      <c r="A49" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B49" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="C49" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="D49" s="2"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B50" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="C50" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="D50" s="2"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B51" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="C51" t="s" s="2">
+        <v>140</v>
+      </c>
+      <c r="D51" s="2"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B52" t="s" s="2">
+        <v>141</v>
+      </c>
+      <c r="C52" t="s" s="2">
+        <v>140</v>
+      </c>
+      <c r="D52" s="2"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B53" t="s" s="2">
+        <v>142</v>
+      </c>
+      <c r="C53" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="D53" s="2"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B54" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="C54" t="s" s="2">
+        <v>145</v>
+      </c>
+      <c r="D54" s="2"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B55" t="s" s="2">
+        <v>146</v>
+      </c>
+      <c r="C55" t="s" s="2">
+        <v>147</v>
+      </c>
+      <c r="D55" s="2"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B56" t="s" s="2">
+        <v>148</v>
+      </c>
+      <c r="C56" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="D56" s="2"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B57" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="C57" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="D57" s="2"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B58" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="C58" t="s" s="2">
+        <v>153</v>
+      </c>
+      <c r="D58" s="2"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B59" t="s" s="2">
+        <v>154</v>
+      </c>
+      <c r="C59" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="D59" s="2"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B60" t="s" s="2">
+        <v>156</v>
+      </c>
+      <c r="C60" t="s" s="2">
+        <v>157</v>
+      </c>
+      <c r="D60" s="2"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B61" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="C61" t="s" s="2">
+        <v>159</v>
+      </c>
+      <c r="D61" s="2"/>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>